<commit_message>
Add test data generation and enhance page object methods for stability
- Implement Exec Maven Plugin to regenerate TestData.xlsx before tests
- Improve waitAndClick and waitAndType methods with retry logic and error handling
- Update AccountPage and HomePage to utilize new waitAndClickWithRetry method
- Modify ProductListPage to handle product selection more robustly
- Refactor error locators in RegisterPage for better accuracy
- Ensure all tests navigate to the base URL before execution
- Update test data in GenerateTestData for dynamic email generation
</commit_message>
<xml_diff>
--- a/Part_A/tutorialsninja-automation/src/test/resources/testdata/TestData.xlsx
+++ b/Part_A/tutorialsninja-automation/src/test/resources/testdata/TestData.xlsx
@@ -43,7 +43,7 @@
     <t>Doe</t>
   </si>
   <si>
-    <t>johndoe_auto1@test.com</t>
+    <t>john_1777548876879@test.com</t>
   </si>
   <si>
     <t>0501234567</t>
@@ -58,7 +58,7 @@
     <t>Smith</t>
   </si>
   <si>
-    <t>janesmith_auto2@test.com</t>
+    <t>jane_1777548876889@test.com</t>
   </si>
   <si>
     <t>0507654321</t>

</xml_diff>